<commit_message>
Added more treasury ALN filters
</commit_message>
<xml_diff>
--- a/input_single_results.xlsx
+++ b/input_single_results.xlsx
@@ -464,7 +464,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CITY OF DECATUR</t>
+          <t>City Of Decatur</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -474,12 +474,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-CITY_OF_DECATUR-376001308-2023.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_Of_Decatur-376001308-2023.docx</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-CITY_OF_DECATUR-376001308-2023.docx</t>
+          <t>http://localhost:8000/local/mdl/2023/MDL-City_Of_Decatur-376001308-2023.docx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>City of New London, CT</t>
+          <t>City of New London</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -505,12 +505,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_New_London_CT-066001880-2024.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_New_London-066001880-2024.docx</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-City_of_New_London_CT-066001880-2024.docx</t>
+          <t>http://localhost:8000/local/mdl/2024/MDL-City_of_New_London-066001880-2024.docx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -526,7 +526,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>City of Oregon City</t>
+          <t>City of Oregon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -536,12 +536,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_Oregon_City-936002230-2023.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-City_of_Oregon-936002230-2023.docx</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-City_of_Oregon_City-936002230-2023.docx</t>
+          <t>http://localhost:8000/local/mdl/2023/MDL-City_of_Oregon-936002230-2023.docx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -588,7 +588,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>COUNTY OF MARIPOSA</t>
+          <t>County of Mariposa</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-COUNTY_OF_MARIPOSA-946000880-2023.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-County_of_Mariposa-946000880-2023.docx</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-COUNTY_OF_MARIPOSA-946000880-2023.docx</t>
+          <t>http://localhost:8000/local/mdl/2023/MDL-County_of_Mariposa-946000880-2023.docx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GALLATIN COUNTY</t>
+          <t>Gallatin County</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-GALLATIN_COUNTY-816001363-2022.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Gallatin_County-816001363-2022.docx</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2022/MDL-GALLATIN_COUNTY-816001363-2022.docx</t>
+          <t>http://localhost:8000/local/mdl/2022/MDL-Gallatin_County-816001363-2022.docx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Presidio County, Texas</t>
+          <t>Presidio County</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -691,12 +691,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Presidio_County_Texas-746001689-2023.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Presidio_County-746001689-2023.docx</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2023/MDL-Presidio_County_Texas-746001689-2023.docx</t>
+          <t>http://localhost:8000/local/mdl/2023/MDL-Presidio_County-746001689-2023.docx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -743,7 +743,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TOWN OF CHARLTON</t>
+          <t>Town of Charlton</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -753,12 +753,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-TOWN_OF_CHARLTON-046001109-2024.docx</t>
+          <t>D:\Documents\Profesh\Forward Edge AI\Treasury AI\single-finding-fix\mdl-backend-demo\outputs\MDL-Town_of_Charlton-046001109-2024.docx</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>http://localhost:8000/local/mdl/2024/MDL-TOWN_OF_CHARLTON-046001109-2024.docx</t>
+          <t>http://localhost:8000/local/mdl/2024/MDL-Town_of_Charlton-046001109-2024.docx</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>

</xml_diff>